<commit_message>
Fixed dropdown auto fill
</commit_message>
<xml_diff>
--- a/pages/video_analysis/IP_Master_Women.xlsx
+++ b/pages/video_analysis/IP_Master_Women.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sportnzgroup-my.sharepoint.com/personal/anja_kuys_hpsnz_org_nz/Documents/Desktop/Scripts/CNZPD/pages/video_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_895A468780AFE1A16BBC3229C9E314422081DEFC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A59DB67-EAE6-4B0A-949F-2DAEC2BC9915}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_AFAA658680BF63C7274CA376ADE30E422081DE5F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE9766A7-B058-404D-8BF5-19940765D433}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1620" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="21">
   <si>
     <t>Title</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t>26-07-31 Glasgow CWG Shearman Q</t>
+  </si>
+  <si>
+    <t>26-07-31 Glasgow CWG Botha F</t>
   </si>
 </sst>
 </file>
@@ -424,10 +427,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I321"/>
+  <dimension ref="A1:I385"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="41.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.9140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
@@ -7825,6 +7834,1478 @@
         <v>9</v>
       </c>
       <c r="I321" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="322" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A322" t="s">
+        <v>20</v>
+      </c>
+      <c r="C322">
+        <v>62.5</v>
+      </c>
+      <c r="D322">
+        <v>9.5199979999999993</v>
+      </c>
+      <c r="E322">
+        <v>9.5199980000000011</v>
+      </c>
+      <c r="F322">
+        <v>23.63445875</v>
+      </c>
+      <c r="G322" t="s">
+        <v>9</v>
+      </c>
+      <c r="I322" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="323" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A323" t="s">
+        <v>20</v>
+      </c>
+      <c r="C323">
+        <v>125</v>
+      </c>
+      <c r="D323">
+        <v>14.732263</v>
+      </c>
+      <c r="E323">
+        <v>5.2122649999999986</v>
+      </c>
+      <c r="F323">
+        <v>43.167413779999997</v>
+      </c>
+      <c r="G323" t="s">
+        <v>9</v>
+      </c>
+      <c r="I323" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="324" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A324" t="s">
+        <v>20</v>
+      </c>
+      <c r="C324">
+        <v>187.5</v>
+      </c>
+      <c r="D324">
+        <v>19.240527</v>
+      </c>
+      <c r="E324">
+        <v>4.5082640000000005</v>
+      </c>
+      <c r="F324">
+        <v>49.908346100000003</v>
+      </c>
+      <c r="G324" t="s">
+        <v>9</v>
+      </c>
+      <c r="I324" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="325" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A325" t="s">
+        <v>20</v>
+      </c>
+      <c r="C325">
+        <v>250</v>
+      </c>
+      <c r="D325">
+        <v>23.516403</v>
+      </c>
+      <c r="E325">
+        <v>4.2758759999999967</v>
+      </c>
+      <c r="F325">
+        <v>52.620796300000002</v>
+      </c>
+      <c r="G325" t="s">
+        <v>9</v>
+      </c>
+      <c r="I325" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="326" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A326" t="s">
+        <v>20</v>
+      </c>
+      <c r="C326">
+        <v>312.5</v>
+      </c>
+      <c r="D326">
+        <v>27.648592000000001</v>
+      </c>
+      <c r="E326">
+        <v>4.1321890000000039</v>
+      </c>
+      <c r="F326">
+        <v>54.450558770000001</v>
+      </c>
+      <c r="G326" t="s">
+        <v>9</v>
+      </c>
+      <c r="I326" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="327" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A327" t="s">
+        <v>20</v>
+      </c>
+      <c r="C327">
+        <v>375</v>
+      </c>
+      <c r="D327">
+        <v>31.713542</v>
+      </c>
+      <c r="E327">
+        <v>4.0649499999999961</v>
+      </c>
+      <c r="F327">
+        <v>55.351234329999997</v>
+      </c>
+      <c r="G327" t="s">
+        <v>9</v>
+      </c>
+      <c r="I327" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="328" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A328" t="s">
+        <v>20</v>
+      </c>
+      <c r="C328">
+        <v>437.5</v>
+      </c>
+      <c r="D328">
+        <v>35.773541999999999</v>
+      </c>
+      <c r="E328">
+        <v>4.0600000000000023</v>
+      </c>
+      <c r="F328">
+        <v>55.418719209999999</v>
+      </c>
+      <c r="G328" t="s">
+        <v>9</v>
+      </c>
+      <c r="I328" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="329" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A329" t="s">
+        <v>20</v>
+      </c>
+      <c r="C329">
+        <v>500</v>
+      </c>
+      <c r="D329">
+        <v>39.793542000000002</v>
+      </c>
+      <c r="E329">
+        <v>4.0200000000000031</v>
+      </c>
+      <c r="F329">
+        <v>55.970149249999999</v>
+      </c>
+      <c r="G329" t="s">
+        <v>9</v>
+      </c>
+      <c r="I329" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="330" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A330" t="s">
+        <v>20</v>
+      </c>
+      <c r="C330">
+        <v>562.5</v>
+      </c>
+      <c r="D330">
+        <v>43.793542000000002</v>
+      </c>
+      <c r="E330">
+        <v>4</v>
+      </c>
+      <c r="F330">
+        <v>56.25</v>
+      </c>
+      <c r="G330" t="s">
+        <v>9</v>
+      </c>
+      <c r="I330" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="331" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A331" t="s">
+        <v>20</v>
+      </c>
+      <c r="C331">
+        <v>625</v>
+      </c>
+      <c r="D331">
+        <v>47.817993999999999</v>
+      </c>
+      <c r="E331">
+        <v>4.0244519999999966</v>
+      </c>
+      <c r="F331">
+        <v>55.90823297</v>
+      </c>
+      <c r="G331" t="s">
+        <v>9</v>
+      </c>
+      <c r="I331" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="332" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A332" t="s">
+        <v>20</v>
+      </c>
+      <c r="C332">
+        <v>687.5</v>
+      </c>
+      <c r="D332">
+        <v>51.837992</v>
+      </c>
+      <c r="E332">
+        <v>4.0199980000000011</v>
+      </c>
+      <c r="F332">
+        <v>55.970177100000001</v>
+      </c>
+      <c r="G332" t="s">
+        <v>9</v>
+      </c>
+      <c r="I332" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="333" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A333" t="s">
+        <v>20</v>
+      </c>
+      <c r="C333">
+        <v>750</v>
+      </c>
+      <c r="D333">
+        <v>55.897981999999999</v>
+      </c>
+      <c r="E333">
+        <v>4.0599899999999991</v>
+      </c>
+      <c r="F333">
+        <v>55.418855710000003</v>
+      </c>
+      <c r="G333" t="s">
+        <v>9</v>
+      </c>
+      <c r="I333" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="334" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A334" t="s">
+        <v>20</v>
+      </c>
+      <c r="C334">
+        <v>812.5</v>
+      </c>
+      <c r="D334">
+        <v>59.937975999999999</v>
+      </c>
+      <c r="E334">
+        <v>4.0399940000000072</v>
+      </c>
+      <c r="F334">
+        <v>55.693152019999999</v>
+      </c>
+      <c r="G334" t="s">
+        <v>9</v>
+      </c>
+      <c r="I334" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="335" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A335" t="s">
+        <v>20</v>
+      </c>
+      <c r="C335">
+        <v>875</v>
+      </c>
+      <c r="D335">
+        <v>64.037968000000006</v>
+      </c>
+      <c r="E335">
+        <v>4.0999920000000003</v>
+      </c>
+      <c r="F335">
+        <v>54.87815586</v>
+      </c>
+      <c r="G335" t="s">
+        <v>9</v>
+      </c>
+      <c r="I335" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="336" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A336" t="s">
+        <v>20</v>
+      </c>
+      <c r="C336">
+        <v>937.5</v>
+      </c>
+      <c r="D336">
+        <v>68.097962999999993</v>
+      </c>
+      <c r="E336">
+        <v>4.0599950000000007</v>
+      </c>
+      <c r="F336">
+        <v>55.418787459999997</v>
+      </c>
+      <c r="G336" t="s">
+        <v>9</v>
+      </c>
+      <c r="I336" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="337" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A337" t="s">
+        <v>20</v>
+      </c>
+      <c r="C337">
+        <v>1000</v>
+      </c>
+      <c r="D337">
+        <v>72.217956999999998</v>
+      </c>
+      <c r="E337">
+        <v>4.1199939999999913</v>
+      </c>
+      <c r="F337">
+        <v>54.611730020000003</v>
+      </c>
+      <c r="G337" t="s">
+        <v>9</v>
+      </c>
+      <c r="I337" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="338" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A338" t="s">
+        <v>20</v>
+      </c>
+      <c r="C338">
+        <v>1062.5</v>
+      </c>
+      <c r="D338">
+        <v>76.297951999999995</v>
+      </c>
+      <c r="E338">
+        <v>4.0799949999999967</v>
+      </c>
+      <c r="F338">
+        <v>55.147126409999998</v>
+      </c>
+      <c r="G338" t="s">
+        <v>9</v>
+      </c>
+      <c r="I338" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="339" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A339" t="s">
+        <v>20</v>
+      </c>
+      <c r="C339">
+        <v>1125</v>
+      </c>
+      <c r="D339">
+        <v>80.397945000000007</v>
+      </c>
+      <c r="E339">
+        <v>4.099993000000012</v>
+      </c>
+      <c r="F339">
+        <v>54.87814247</v>
+      </c>
+      <c r="G339" t="s">
+        <v>9</v>
+      </c>
+      <c r="I339" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="340" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A340" t="s">
+        <v>20</v>
+      </c>
+      <c r="C340">
+        <v>1187.5</v>
+      </c>
+      <c r="D340">
+        <v>84.497936999999993</v>
+      </c>
+      <c r="E340">
+        <v>4.0999919999999861</v>
+      </c>
+      <c r="F340">
+        <v>54.87815586</v>
+      </c>
+      <c r="G340" t="s">
+        <v>9</v>
+      </c>
+      <c r="I340" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="341" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A341" t="s">
+        <v>20</v>
+      </c>
+      <c r="C341">
+        <v>1250</v>
+      </c>
+      <c r="D341">
+        <v>88.577934999999997</v>
+      </c>
+      <c r="E341">
+        <v>4.0799980000000033</v>
+      </c>
+      <c r="F341">
+        <v>55.147085859999997</v>
+      </c>
+      <c r="G341" t="s">
+        <v>9</v>
+      </c>
+      <c r="I341" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="342" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A342" t="s">
+        <v>20</v>
+      </c>
+      <c r="C342">
+        <v>1312.5</v>
+      </c>
+      <c r="D342">
+        <v>92.637932000000006</v>
+      </c>
+      <c r="E342">
+        <v>4.0599970000000098</v>
+      </c>
+      <c r="F342">
+        <v>55.418760159999998</v>
+      </c>
+      <c r="G342" t="s">
+        <v>9</v>
+      </c>
+      <c r="I342" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="343" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A343" t="s">
+        <v>20</v>
+      </c>
+      <c r="C343">
+        <v>1375</v>
+      </c>
+      <c r="D343">
+        <v>96.717930999999993</v>
+      </c>
+      <c r="E343">
+        <v>4.0799990000000008</v>
+      </c>
+      <c r="F343">
+        <v>55.147072340000001</v>
+      </c>
+      <c r="G343" t="s">
+        <v>9</v>
+      </c>
+      <c r="I343" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="344" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A344" t="s">
+        <v>20</v>
+      </c>
+      <c r="C344">
+        <v>1437.5</v>
+      </c>
+      <c r="D344">
+        <v>100.79792999999999</v>
+      </c>
+      <c r="E344">
+        <v>4.0799989999999866</v>
+      </c>
+      <c r="F344">
+        <v>55.147072340000001</v>
+      </c>
+      <c r="G344" t="s">
+        <v>9</v>
+      </c>
+      <c r="I344" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="345" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A345" t="s">
+        <v>20</v>
+      </c>
+      <c r="C345">
+        <v>1500</v>
+      </c>
+      <c r="D345">
+        <v>104.89792799999999</v>
+      </c>
+      <c r="E345">
+        <v>4.0999979999999994</v>
+      </c>
+      <c r="F345">
+        <v>54.878075549999998</v>
+      </c>
+      <c r="G345" t="s">
+        <v>9</v>
+      </c>
+      <c r="I345" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="346" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A346" t="s">
+        <v>20</v>
+      </c>
+      <c r="C346">
+        <v>1562.5</v>
+      </c>
+      <c r="D346">
+        <v>108.977926</v>
+      </c>
+      <c r="E346">
+        <v>4.0799980000000033</v>
+      </c>
+      <c r="F346">
+        <v>55.147085859999997</v>
+      </c>
+      <c r="G346" t="s">
+        <v>9</v>
+      </c>
+      <c r="I346" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="347" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A347" t="s">
+        <v>20</v>
+      </c>
+      <c r="C347">
+        <v>1625</v>
+      </c>
+      <c r="D347">
+        <v>113.057923</v>
+      </c>
+      <c r="E347">
+        <v>4.0799970000000059</v>
+      </c>
+      <c r="F347">
+        <v>55.147099369999999</v>
+      </c>
+      <c r="G347" t="s">
+        <v>9</v>
+      </c>
+      <c r="I347" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="348" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A348" t="s">
+        <v>20</v>
+      </c>
+      <c r="C348">
+        <v>1687.5</v>
+      </c>
+      <c r="D348">
+        <v>117.137922</v>
+      </c>
+      <c r="E348">
+        <v>4.0799990000000008</v>
+      </c>
+      <c r="F348">
+        <v>55.147072340000001</v>
+      </c>
+      <c r="G348" t="s">
+        <v>9</v>
+      </c>
+      <c r="I348" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="349" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A349" t="s">
+        <v>20</v>
+      </c>
+      <c r="C349">
+        <v>1750</v>
+      </c>
+      <c r="D349">
+        <v>121.217921</v>
+      </c>
+      <c r="E349">
+        <v>4.0799989999999866</v>
+      </c>
+      <c r="F349">
+        <v>55.147072340000001</v>
+      </c>
+      <c r="G349" t="s">
+        <v>9</v>
+      </c>
+      <c r="I349" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="350" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A350" t="s">
+        <v>20</v>
+      </c>
+      <c r="C350">
+        <v>1812.5</v>
+      </c>
+      <c r="D350">
+        <v>125.297921</v>
+      </c>
+      <c r="E350">
+        <v>4.0800000000000125</v>
+      </c>
+      <c r="F350">
+        <v>55.147058819999998</v>
+      </c>
+      <c r="G350" t="s">
+        <v>9</v>
+      </c>
+      <c r="I350" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="351" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A351" t="s">
+        <v>20</v>
+      </c>
+      <c r="C351">
+        <v>1875</v>
+      </c>
+      <c r="D351">
+        <v>129.397921</v>
+      </c>
+      <c r="E351">
+        <v>4.0999999999999943</v>
+      </c>
+      <c r="F351">
+        <v>54.87804878</v>
+      </c>
+      <c r="G351" t="s">
+        <v>9</v>
+      </c>
+      <c r="I351" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="352" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A352" t="s">
+        <v>20</v>
+      </c>
+      <c r="C352">
+        <v>1937.5</v>
+      </c>
+      <c r="D352">
+        <v>133.47792000000001</v>
+      </c>
+      <c r="E352">
+        <v>4.079999000000015</v>
+      </c>
+      <c r="F352">
+        <v>55.147072340000001</v>
+      </c>
+      <c r="G352" t="s">
+        <v>9</v>
+      </c>
+      <c r="I352" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="353" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A353" t="s">
+        <v>20</v>
+      </c>
+      <c r="C353">
+        <v>2000</v>
+      </c>
+      <c r="D353">
+        <v>137.57792000000001</v>
+      </c>
+      <c r="E353">
+        <v>4.0999999999999943</v>
+      </c>
+      <c r="F353">
+        <v>54.87804878</v>
+      </c>
+      <c r="G353" t="s">
+        <v>9</v>
+      </c>
+      <c r="I353" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="354" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A354" t="s">
+        <v>20</v>
+      </c>
+      <c r="C354">
+        <v>2062.5</v>
+      </c>
+      <c r="D354">
+        <v>141.65791999999999</v>
+      </c>
+      <c r="E354">
+        <v>4.0799999999999841</v>
+      </c>
+      <c r="F354">
+        <v>55.147058819999998</v>
+      </c>
+      <c r="G354" t="s">
+        <v>9</v>
+      </c>
+      <c r="I354" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="355" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A355" t="s">
+        <v>20</v>
+      </c>
+      <c r="C355">
+        <v>2125</v>
+      </c>
+      <c r="D355">
+        <v>145.77791999999999</v>
+      </c>
+      <c r="E355">
+        <v>4.1200000000000045</v>
+      </c>
+      <c r="F355">
+        <v>54.611650490000002</v>
+      </c>
+      <c r="G355" t="s">
+        <v>9</v>
+      </c>
+      <c r="I355" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="356" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A356" t="s">
+        <v>20</v>
+      </c>
+      <c r="C356">
+        <v>2187.5</v>
+      </c>
+      <c r="D356">
+        <v>149.89792</v>
+      </c>
+      <c r="E356">
+        <v>4.1200000000000045</v>
+      </c>
+      <c r="F356">
+        <v>54.611650490000002</v>
+      </c>
+      <c r="G356" t="s">
+        <v>9</v>
+      </c>
+      <c r="I356" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="357" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A357" t="s">
+        <v>20</v>
+      </c>
+      <c r="C357">
+        <v>2250</v>
+      </c>
+      <c r="D357">
+        <v>153.99791999999999</v>
+      </c>
+      <c r="E357">
+        <v>4.0999999999999943</v>
+      </c>
+      <c r="F357">
+        <v>54.87804878</v>
+      </c>
+      <c r="G357" t="s">
+        <v>9</v>
+      </c>
+      <c r="I357" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="358" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A358" t="s">
+        <v>20</v>
+      </c>
+      <c r="C358">
+        <v>2312.5</v>
+      </c>
+      <c r="D358">
+        <v>158.09791999999999</v>
+      </c>
+      <c r="E358">
+        <v>4.0999999999999943</v>
+      </c>
+      <c r="F358">
+        <v>54.87804878</v>
+      </c>
+      <c r="G358" t="s">
+        <v>9</v>
+      </c>
+      <c r="I358" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="359" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A359" t="s">
+        <v>20</v>
+      </c>
+      <c r="C359">
+        <v>2375</v>
+      </c>
+      <c r="D359">
+        <v>162.21791999999999</v>
+      </c>
+      <c r="E359">
+        <v>4.1200000000000045</v>
+      </c>
+      <c r="F359">
+        <v>54.611650490000002</v>
+      </c>
+      <c r="G359" t="s">
+        <v>9</v>
+      </c>
+      <c r="I359" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="360" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A360" t="s">
+        <v>20</v>
+      </c>
+      <c r="C360">
+        <v>2437.5</v>
+      </c>
+      <c r="D360">
+        <v>166.33792</v>
+      </c>
+      <c r="E360">
+        <v>4.1200000000000045</v>
+      </c>
+      <c r="F360">
+        <v>54.611650490000002</v>
+      </c>
+      <c r="G360" t="s">
+        <v>9</v>
+      </c>
+      <c r="I360" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="361" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A361" t="s">
+        <v>20</v>
+      </c>
+      <c r="C361">
+        <v>2500</v>
+      </c>
+      <c r="D361">
+        <v>170.47792000000001</v>
+      </c>
+      <c r="E361">
+        <v>4.1400000000000148</v>
+      </c>
+      <c r="F361">
+        <v>54.347826089999998</v>
+      </c>
+      <c r="G361" t="s">
+        <v>9</v>
+      </c>
+      <c r="I361" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="362" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A362" t="s">
+        <v>20</v>
+      </c>
+      <c r="C362">
+        <v>2562.5</v>
+      </c>
+      <c r="D362">
+        <v>174.61792</v>
+      </c>
+      <c r="E362">
+        <v>4.1399999999999864</v>
+      </c>
+      <c r="F362">
+        <v>54.347826089999998</v>
+      </c>
+      <c r="G362" t="s">
+        <v>9</v>
+      </c>
+      <c r="I362" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="363" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A363" t="s">
+        <v>20</v>
+      </c>
+      <c r="C363">
+        <v>2625</v>
+      </c>
+      <c r="D363">
+        <v>178.73792</v>
+      </c>
+      <c r="E363">
+        <v>4.1200000000000045</v>
+      </c>
+      <c r="F363">
+        <v>54.611650490000002</v>
+      </c>
+      <c r="G363" t="s">
+        <v>9</v>
+      </c>
+      <c r="I363" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="364" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A364" t="s">
+        <v>20</v>
+      </c>
+      <c r="C364">
+        <v>2687.5</v>
+      </c>
+      <c r="D364">
+        <v>182.87791999999999</v>
+      </c>
+      <c r="E364">
+        <v>4.1399999999999864</v>
+      </c>
+      <c r="F364">
+        <v>54.347826089999998</v>
+      </c>
+      <c r="G364" t="s">
+        <v>9</v>
+      </c>
+      <c r="I364" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="365" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A365" t="s">
+        <v>20</v>
+      </c>
+      <c r="C365">
+        <v>2750</v>
+      </c>
+      <c r="D365">
+        <v>187.01792</v>
+      </c>
+      <c r="E365">
+        <v>4.1400000000000148</v>
+      </c>
+      <c r="F365">
+        <v>54.347826089999998</v>
+      </c>
+      <c r="G365" t="s">
+        <v>9</v>
+      </c>
+      <c r="I365" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="366" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A366" t="s">
+        <v>20</v>
+      </c>
+      <c r="C366">
+        <v>2812.5</v>
+      </c>
+      <c r="D366">
+        <v>191.17792</v>
+      </c>
+      <c r="E366">
+        <v>4.1599999999999966</v>
+      </c>
+      <c r="F366">
+        <v>54.08653846</v>
+      </c>
+      <c r="G366" t="s">
+        <v>9</v>
+      </c>
+      <c r="I366" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="367" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A367" t="s">
+        <v>20</v>
+      </c>
+      <c r="C367">
+        <v>2875</v>
+      </c>
+      <c r="D367">
+        <v>195.33792</v>
+      </c>
+      <c r="E367">
+        <v>4.1599999999999966</v>
+      </c>
+      <c r="F367">
+        <v>54.08653846</v>
+      </c>
+      <c r="G367" t="s">
+        <v>9</v>
+      </c>
+      <c r="I367" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="368" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A368" t="s">
+        <v>20</v>
+      </c>
+      <c r="C368">
+        <v>2937.5</v>
+      </c>
+      <c r="D368">
+        <v>199.49791999999999</v>
+      </c>
+      <c r="E368">
+        <v>4.1599999999999966</v>
+      </c>
+      <c r="F368">
+        <v>54.08653846</v>
+      </c>
+      <c r="G368" t="s">
+        <v>9</v>
+      </c>
+      <c r="I368" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="369" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A369" t="s">
+        <v>20</v>
+      </c>
+      <c r="C369">
+        <v>3000</v>
+      </c>
+      <c r="D369">
+        <v>203.677919</v>
+      </c>
+      <c r="E369">
+        <v>4.1799990000000093</v>
+      </c>
+      <c r="F369">
+        <v>53.827764070000001</v>
+      </c>
+      <c r="G369" t="s">
+        <v>9</v>
+      </c>
+      <c r="I369" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="370" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A370" t="s">
+        <v>20</v>
+      </c>
+      <c r="C370">
+        <v>3062.5</v>
+      </c>
+      <c r="D370">
+        <v>207.91791900000001</v>
+      </c>
+      <c r="E370">
+        <v>4.2400000000000091</v>
+      </c>
+      <c r="F370">
+        <v>53.066037739999999</v>
+      </c>
+      <c r="G370" t="s">
+        <v>9</v>
+      </c>
+      <c r="I370" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="371" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A371" t="s">
+        <v>20</v>
+      </c>
+      <c r="C371">
+        <v>3125</v>
+      </c>
+      <c r="D371">
+        <v>212.117919</v>
+      </c>
+      <c r="E371">
+        <v>4.1999999999999886</v>
+      </c>
+      <c r="F371">
+        <v>53.571428570000002</v>
+      </c>
+      <c r="G371" t="s">
+        <v>9</v>
+      </c>
+      <c r="I371" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="372" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A372" t="s">
+        <v>20</v>
+      </c>
+      <c r="C372">
+        <v>3187.5</v>
+      </c>
+      <c r="D372">
+        <v>216.337919</v>
+      </c>
+      <c r="E372">
+        <v>4.2199999999999989</v>
+      </c>
+      <c r="F372">
+        <v>53.317535550000002</v>
+      </c>
+      <c r="G372" t="s">
+        <v>9</v>
+      </c>
+      <c r="I372" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="373" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A373" t="s">
+        <v>20</v>
+      </c>
+      <c r="C373">
+        <v>3250</v>
+      </c>
+      <c r="D373">
+        <v>220.557919</v>
+      </c>
+      <c r="E373">
+        <v>4.2199999999999989</v>
+      </c>
+      <c r="F373">
+        <v>53.317535550000002</v>
+      </c>
+      <c r="G373" t="s">
+        <v>9</v>
+      </c>
+      <c r="I373" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="374" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A374" t="s">
+        <v>20</v>
+      </c>
+      <c r="C374">
+        <v>3312.5</v>
+      </c>
+      <c r="D374">
+        <v>224.777919</v>
+      </c>
+      <c r="E374">
+        <v>4.2199999999999989</v>
+      </c>
+      <c r="F374">
+        <v>53.317535550000002</v>
+      </c>
+      <c r="G374" t="s">
+        <v>9</v>
+      </c>
+      <c r="I374" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="375" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A375" t="s">
+        <v>20</v>
+      </c>
+      <c r="C375">
+        <v>3375</v>
+      </c>
+      <c r="D375">
+        <v>228.997919</v>
+      </c>
+      <c r="E375">
+        <v>4.2199999999999989</v>
+      </c>
+      <c r="F375">
+        <v>53.317535550000002</v>
+      </c>
+      <c r="G375" t="s">
+        <v>9</v>
+      </c>
+      <c r="I375" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="376" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A376" t="s">
+        <v>20</v>
+      </c>
+      <c r="C376">
+        <v>3437.5</v>
+      </c>
+      <c r="D376">
+        <v>233.23791900000001</v>
+      </c>
+      <c r="E376">
+        <v>4.2400000000000091</v>
+      </c>
+      <c r="F376">
+        <v>53.066037739999999</v>
+      </c>
+      <c r="G376" t="s">
+        <v>9</v>
+      </c>
+      <c r="I376" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="377" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A377" t="s">
+        <v>20</v>
+      </c>
+      <c r="C377">
+        <v>3500</v>
+      </c>
+      <c r="D377">
+        <v>237.457919</v>
+      </c>
+      <c r="E377">
+        <v>4.2199999999999989</v>
+      </c>
+      <c r="F377">
+        <v>53.317535550000002</v>
+      </c>
+      <c r="G377" t="s">
+        <v>9</v>
+      </c>
+      <c r="I377" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="378" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A378" t="s">
+        <v>20</v>
+      </c>
+      <c r="C378">
+        <v>3562.5</v>
+      </c>
+      <c r="D378">
+        <v>241.69791900000001</v>
+      </c>
+      <c r="E378">
+        <v>4.2400000000000091</v>
+      </c>
+      <c r="F378">
+        <v>53.066037739999999</v>
+      </c>
+      <c r="G378" t="s">
+        <v>9</v>
+      </c>
+      <c r="I378" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="379" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A379" t="s">
+        <v>20</v>
+      </c>
+      <c r="C379">
+        <v>3625</v>
+      </c>
+      <c r="D379">
+        <v>245.95791</v>
+      </c>
+      <c r="E379">
+        <v>4.2599909999999852</v>
+      </c>
+      <c r="F379">
+        <v>52.817012990000002</v>
+      </c>
+      <c r="G379" t="s">
+        <v>9</v>
+      </c>
+      <c r="I379" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="380" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A380" t="s">
+        <v>20</v>
+      </c>
+      <c r="C380">
+        <v>3687.5</v>
+      </c>
+      <c r="D380">
+        <v>250.21789799999999</v>
+      </c>
+      <c r="E380">
+        <v>4.2599880000000212</v>
+      </c>
+      <c r="F380">
+        <v>52.817050190000003</v>
+      </c>
+      <c r="G380" t="s">
+        <v>9</v>
+      </c>
+      <c r="I380" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="381" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A381" t="s">
+        <v>20</v>
+      </c>
+      <c r="C381">
+        <v>3750</v>
+      </c>
+      <c r="D381">
+        <v>254.47788800000001</v>
+      </c>
+      <c r="E381">
+        <v>4.2599899999999593</v>
+      </c>
+      <c r="F381">
+        <v>52.817025389999998</v>
+      </c>
+      <c r="G381" t="s">
+        <v>9</v>
+      </c>
+      <c r="I381" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="382" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A382" t="s">
+        <v>20</v>
+      </c>
+      <c r="C382">
+        <v>3812.5</v>
+      </c>
+      <c r="D382">
+        <v>258.73788300000001</v>
+      </c>
+      <c r="E382">
+        <v>4.2599950000000035</v>
+      </c>
+      <c r="F382">
+        <v>52.816963399999999</v>
+      </c>
+      <c r="G382" t="s">
+        <v>9</v>
+      </c>
+      <c r="I382" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="383" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A383" t="s">
+        <v>20</v>
+      </c>
+      <c r="C383">
+        <v>3875</v>
+      </c>
+      <c r="D383">
+        <v>262.99787900000001</v>
+      </c>
+      <c r="E383">
+        <v>4.259996000000001</v>
+      </c>
+      <c r="F383">
+        <v>52.816951000000003</v>
+      </c>
+      <c r="G383" t="s">
+        <v>9</v>
+      </c>
+      <c r="I383" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="384" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A384" t="s">
+        <v>20</v>
+      </c>
+      <c r="C384">
+        <v>3937.5</v>
+      </c>
+      <c r="D384">
+        <v>267.23787399999998</v>
+      </c>
+      <c r="E384">
+        <v>4.2399950000000217</v>
+      </c>
+      <c r="F384">
+        <v>53.066100310000003</v>
+      </c>
+      <c r="G384" t="s">
+        <v>9</v>
+      </c>
+      <c r="I384" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="385" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A385" t="s">
+        <v>20</v>
+      </c>
+      <c r="C385">
+        <v>4000</v>
+      </c>
+      <c r="D385">
+        <v>271.49786799999998</v>
+      </c>
+      <c r="E385">
+        <v>4.2599940000000061</v>
+      </c>
+      <c r="F385">
+        <v>52.816975800000002</v>
+      </c>
+      <c r="G385" t="s">
+        <v>9</v>
+      </c>
+      <c r="I385" t="s">
         <v>18</v>
       </c>
     </row>
@@ -7837,13 +9318,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I193 A194:A321 I194:I321" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I321 A322:A385 I322:I385" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{9d5ca952-e4a5-43e6-b17c-c01d313ad135}" enabled="0" method="" siteId="{9d5ca952-e4a5-43e6-b17c-c01d313ad135}" removed="1"/>
-</clbl:labelList>
 </file>
</xml_diff>